<commit_message>
Update stocks.xlsx with real positions (5 holdings + 6 watchlist)
</commit_message>
<xml_diff>
--- a/stocks.xlsx
+++ b/stocks.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,10 +451,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>6.58</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>11084</v>
       </c>
     </row>
     <row r="3">
@@ -469,10 +469,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="4">
@@ -487,100 +487,46 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>33.386</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>000960</t>
+          <t>603233</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>锡业股份</t>
+          <t>大参林</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>17.08</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>002714</t>
+          <t>601998</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>牧原股份</t>
+          <t>中信银行</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>8.154</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>600900</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>长江电力</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>600036</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>招商银行</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>601166</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>兴业银行</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
     </row>
   </sheetData>
@@ -594,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -624,12 +570,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>600989</t>
+          <t>000960</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>宝丰能源</t>
+          <t>锡业股份</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>002714</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>牧原股份</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>600900</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>长江电力</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>600036</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>招商银行</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>601166</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>兴业银行</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Feishu webhook cards
</commit_message>
<xml_diff>
--- a/stocks.xlsx
+++ b/stocks.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -557,7 +557,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>601998</t>
         </is>
@@ -569,7 +569,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>000960</t>
         </is>
@@ -581,7 +581,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>002714</t>
         </is>
@@ -593,7 +593,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>600900</t>
         </is>
@@ -605,7 +605,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>600036</t>
         </is>
@@ -617,7 +617,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>601166</t>
         </is>
@@ -737,7 +737,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>002747</t>
         </is>
@@ -749,7 +749,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>002050</t>
         </is>
@@ -757,6 +757,42 @@
       <c r="B18" t="inlineStr">
         <is>
           <t>三花智控</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>601328</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>交通银行</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>601088</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>中国神华</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>600584</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>长电科技</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: support Hong Kong watchlist quotes
</commit_message>
<xml_diff>
--- a/stocks.xlsx
+++ b/stocks.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,6 +796,114 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>300760</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>迈瑞医疗</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>600276</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>恒瑞医药</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>688235</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>百济神州</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>688617</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>惠泰医疗</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>688271</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>联影医疗</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>002223</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>鱼跃医疗</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>HK01801</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>信达生物</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HK09926</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>康方生物</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HK02269</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>药明生物</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update watchlist holdings
</commit_message>
<xml_diff>
--- a/stocks.xlsx
+++ b/stocks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="portfolio" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="watchlist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="portfolio" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="watchlist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -904,6 +904,138 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>002371</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>北方华创</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>688012</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>中微公司</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>688072</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>拓荆科技</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>688120</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>华海清科</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>003816</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>中国广核</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>601985</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>中国核电</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>002837</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>英维克</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>301018</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>申菱环境</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>300990</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>同飞股份</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>688041</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>海光信息</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>688256</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>寒武纪</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>